<commit_message>
AR Work bench changes
</commit_message>
<xml_diff>
--- a/docs/Denial_WorkFlow/ARWorkflow_Redesign_Plan_v1.0_09.25.2026.xlsx
+++ b/docs/Denial_WorkFlow/ARWorkflow_Redesign_Plan_v1.0_09.25.2026.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plan'!$B$3:$L$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Plan - Corrected Order'!$B$5:$N$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Plan - Corrected Order'!$B$5:$P$87</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,10 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
-  <fonts count="24">
+  <numFmts count="0"/>
+  <fonts count="26">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -182,6 +180,16 @@
       <color rgb="FFC00000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -275,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -464,10 +472,78 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -5316,7 +5392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N92"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5333,6 +5409,8 @@
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="70" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="70" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5443,6 +5521,16 @@
           <t>Change &amp; Reason</t>
         </is>
       </c>
+      <c r="O5" s="17" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="P5" s="17" t="inlineStr">
+        <is>
+          <t>Status Notes (AR Workbench)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="64" t="n">
@@ -5502,6 +5590,16 @@
           <t>No change. Close D-01 … D-17 here: D-03 (primary category), D-04 / D-08 (recovery logic) and D-05 / D-06 (claim closure) change the data model and the queue engine built next.</t>
         </is>
       </c>
+      <c r="O6" s="76" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P6" s="77" t="inlineStr">
+        <is>
+          <t>Clarifications sheet: only D-01 and D-03 have a decision; D-02, D-04 … D-17 are still open.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="68" t="n">
@@ -5561,6 +5659,16 @@
           <t>Moved from P2 (was after Follow-Up Management). Every screen's menu, route guard and API check reads the permission matrix, and My Work's own-caseload rule needs the agent role — building the screens first means going back to each one.</t>
         </is>
       </c>
+      <c r="O7" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P7" s="77" t="inlineStr">
+        <is>
+          <t>8 'AR Workbench - …' roles + RoleFeatureAccess matrix (LRNMaster_01_ARWB_Roles_Access.sql); every API call checks the permission.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="68" t="n">
@@ -5620,6 +5728,16 @@
           <t>Moved from P2 with T049. Module ID was a duplicate M11 (also used by Follow-Up Management).</t>
         </is>
       </c>
+      <c r="O8" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P8" s="77" t="inlineStr">
+        <is>
+          <t>navigation.js drives the sidebar and the route guard; API enforces the same roles.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="68" t="n">
@@ -5679,6 +5797,16 @@
           <t>Moved from P2. The scoped-claims filter has to be in every query, export and report from the first one; adding it after the screens exist means revisiting every query.</t>
         </is>
       </c>
+      <c r="O9" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P9" s="77" t="inlineStr">
+        <is>
+          <t>Clinic / provider / agent scope applied in SQL on every claim query (SqlArWorkbenchRepository.AppendScope).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="68" t="n">
@@ -5738,6 +5866,16 @@
           <t>Moved from P2 with T051.</t>
         </is>
       </c>
+      <c r="O10" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P10" s="77" t="inlineStr">
+        <is>
+          <t>Scope badge in the top bar for clinic / provider-scoped users (AppShell).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="68" t="n">
@@ -5797,6 +5935,16 @@
           <t>Moved ahead of the data sync: the sync and the queue engine read these masters.</t>
         </is>
       </c>
+      <c r="O11" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P11" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: Denial Categories (add / edit / deactivate / delete).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="68" t="n">
@@ -5856,6 +6004,16 @@
           <t>Moved ahead of the data sync. TFL thresholds are read by T040.</t>
         </is>
       </c>
+      <c r="O12" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P12" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Timely Filing Limits: limit per financial class, default limit and risk window; saving recalculates every claim's TFL deadline and risk flag.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="68" t="n">
@@ -5915,6 +6073,16 @@
           <t>Moved ahead of the data sync: the Non-Collectible list drives the Non-Collectible sub-queues (T035) and Automatic Adjustment (T033).</t>
         </is>
       </c>
+      <c r="O13" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P13" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: Non-Collectible Denial Codes.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="68" t="n">
@@ -5974,6 +6142,16 @@
           <t>Moved ahead of the data sync.</t>
         </is>
       </c>
+      <c r="O14" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P14" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: Claim Types, Follow-Up Types, Follow-Up Claim Statuses.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="68" t="n">
@@ -6033,6 +6211,16 @@
           <t>Moved ahead of the data sync.</t>
         </is>
       </c>
+      <c r="O15" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P15" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: Panel Types.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="68" t="n">
@@ -6092,6 +6280,16 @@
           <t>Moved ahead of the data sync.</t>
         </is>
       </c>
+      <c r="O16" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P16" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: Denial Root Cause Options.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="68" t="n">
@@ -6151,6 +6349,16 @@
           <t>Moved ahead of the data sync.</t>
         </is>
       </c>
+      <c r="O17" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P17" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: Fix / Resolution Options. Fix / Resolution by Status is view-only.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="68" t="n">
@@ -6210,6 +6418,16 @@
           <t>Moved ahead of the data sync: the sync sets each claim's denial category from this map.</t>
         </is>
       </c>
+      <c r="O18" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P18" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Denial Code Master (Super Master) and Workbench Category Map, with Excel import / export and Apply to claims.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="68" t="n">
@@ -6269,6 +6487,16 @@
           <t>Moved ahead of the data sync.</t>
         </is>
       </c>
+      <c r="O19" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P19" s="77" t="inlineStr">
+        <is>
+          <t>Master Values &gt; Workbench Lists: CIP Categories, CIP Required Information.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="68" t="n">
@@ -6328,6 +6556,16 @@
           <t>Moved here from Log Follow-Up Note. DUPLICATE of T015 / T017 / T018 / T020 (the same Comments Framework masters) — merge and drop one estimate.</t>
         </is>
       </c>
+      <c r="O20" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P20" s="77" t="inlineStr">
+        <is>
+          <t>Same masters as T015 / T017 / T018 / T020 (duplicate task).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="68" t="n">
@@ -6387,6 +6625,16 @@
           <t>Moved before the AR claim table and sync (was after the Work Queue). The financial and recovery columns belong in the AR claim table (T002); adding them after the sync is built means changing the table and the sync twice.</t>
         </is>
       </c>
+      <c r="O21" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P21" s="77" t="inlineStr">
+        <is>
+          <t>Financial &amp; recovery columns on dbo.ARWB_Claim (initial AR, revenue expectation, variance, underpayment, recovered, remaining AR).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="68" t="n">
@@ -6446,6 +6694,16 @@
           <t>Moved before the data sync: the sync writes the 'Claim Identified' / 'Source Data Updated' activity rows, and every later screen writes to these tables.</t>
         </is>
       </c>
+      <c r="O22" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P22" s="77" t="inlineStr">
+        <is>
+          <t>Tables: ARWB_ClaimActivity, ClaimFollowUp, ClaimQaReview, AgentRequest, CipCase(+History), Document.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="64" t="n">
@@ -6505,6 +6763,16 @@
           <t>No change in order within the module; now after the data model and masters it depends on.</t>
         </is>
       </c>
+      <c r="O23" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P23" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_Claim + ARWB_ClaimLine + ARWB_ClaimLineDenial.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="64" t="n">
@@ -6561,6 +6829,16 @@
         </is>
       </c>
       <c r="N24" s="65" t="inlineStr"/>
+      <c r="O24" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P24" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_usp_LoadClaimsFromSource syncs every claim and line, then classifies them.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="64" t="n">
@@ -6617,6 +6895,16 @@
         </is>
       </c>
       <c r="N25" s="65" t="inlineStr"/>
+      <c r="O25" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P25" s="77" t="inlineStr">
+        <is>
+          <t>Claim workspace tabs: Overview, CPT / Line Details, Denial, Follow-Ups, Activity Timeline.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="64" t="n">
@@ -6672,6 +6960,16 @@
         </is>
       </c>
       <c r="N26" s="65" t="inlineStr"/>
+      <c r="O26" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P26" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_DenialInsight + ARWB_DenialInsightClaim.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="64" t="n">
@@ -6728,6 +7026,16 @@
         </is>
       </c>
       <c r="N27" s="65" t="inlineStr"/>
+      <c r="O27" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P27" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_usp_BuildDenialInsights builds current + previous week insights from the synced claims (not copied from the Denial Summary report).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="64" t="n">
@@ -6783,6 +7091,16 @@
         </is>
       </c>
       <c r="N28" s="65" t="inlineStr"/>
+      <c r="O28" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P28" s="77" t="inlineStr">
+        <is>
+          <t>Insights stored per refresh run / sync week (dbo.ARWB_vw_DenialInsight).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="64" t="n">
@@ -6838,6 +7156,16 @@
         </is>
       </c>
       <c r="N29" s="65" t="inlineStr"/>
+      <c r="O29" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P29" s="77" t="inlineStr">
+        <is>
+          <t>Run Data Processing runs the sync, which rebuilds the insights (step 5 of the load procedure).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="68" t="n">
@@ -6897,6 +7225,16 @@
           <t>Moved here from the Financial &amp; Recovery Data Model: the weekly payment / AR refresh runs inside the same weekly sync.</t>
         </is>
       </c>
+      <c r="O30" s="76" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P30" s="77" t="inlineStr">
+        <is>
+          <t>Weekly sync refreshes payments and balances; recovery attribution rule ('payment after first AR activity') waits on decision D-08.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="64" t="n">
@@ -6952,6 +7290,16 @@
         </is>
       </c>
       <c r="N31" s="65" t="inlineStr"/>
+      <c r="O31" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P31" s="77" t="inlineStr">
+        <is>
+          <t>Data Processing screen: run history, last refresh, source period, record counts, Run Data Processing.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="68" t="n">
@@ -7011,6 +7359,16 @@
           <t>Moved before the Work Queue (was after it): the grid's Aging, TFL, Priority and AR Queue columns (T022) come from these rules.</t>
         </is>
       </c>
+      <c r="O32" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P32" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_usp_RecalculateClaimState: financially closed, work complete, open insurance AR, re-follow-up due, follow-up actionable.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="68" t="n">
@@ -7070,6 +7428,16 @@
           <t>Moved before the Work Queue.</t>
         </is>
       </c>
+      <c r="O33" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P33" s="77" t="inlineStr">
+        <is>
+          <t>Queue engine in the same procedure: 12 AR queues + collectible / non-collectible sub-queues from dbo.ARWB_ArQueue.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="68" t="n">
@@ -7129,6 +7497,16 @@
           <t>Moved before the Work Queue and the follow-up note, which move claims through these statuses.</t>
         </is>
       </c>
+      <c r="O34" s="76" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P34" s="77" t="inlineStr">
+        <is>
+          <t>Assignment (Unassigned/Completed -&gt; Assigned) and follow-up (-&gt; Submitted for QA, QA review Awaiting QA, CIP case Awaiting QA) transitions done; QA approve/reject and CIP transitions not built.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="68" t="n">
@@ -7188,6 +7566,16 @@
           <t>Moved here from Workflow Event &amp; Snapshot Infrastructure. DUPLICATE of T040 (same text) — merge and drop one estimate.</t>
         </is>
       </c>
+      <c r="O35" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P35" s="77" t="inlineStr">
+        <is>
+          <t>Same as T040 (duplicate task).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="68" t="n">
@@ -7247,6 +7635,16 @@
           <t>Moved before the Work Queue: TFL is a Work Queue column and filter.</t>
         </is>
       </c>
+      <c r="O36" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P36" s="77" t="inlineStr">
+        <is>
+          <t>TflDeadline / IsTflRisk computed per claim; TFL column and 'TFL risk only' filter on the Work Queue.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="68" t="n">
@@ -7307,6 +7705,16 @@
           <t>Moved after the queue engine (was listed before it). It acts on the Non-Collectible sub-queues from T035 and writes its System / Automation audit entry to T037.</t>
         </is>
       </c>
+      <c r="O37" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P37" s="77" t="inlineStr">
+        <is>
+          <t>API POST /api/ar-workbench/auto-adjustments/preview|process|mark-posted over ARWB_usp_ProcessAutoAdjustments / MarkAdjustmentsPosted (System Admin / RCM Manager / Team Lead). Work Queue: Process Automatic Adjustments (selected or all eligible) with count/$ confirmation, Mark as Posted for selected. Claim page: single Process Automatic Adjustment + Mark as Posted. System / Automation activity entry written by the procedure. Open item: AutoAdjustIncludesNonCollectible = 0, so only AUTO_ADJUST_CODE codes are eligible until set to 1.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="68" t="n">
@@ -7366,6 +7774,16 @@
           <t>Kept in P1, after the queue engine: the nightly snapshot stores each claim's AR queue. Start it early so trend history exists by the P4 reports.</t>
         </is>
       </c>
+      <c r="O38" s="76" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P38" s="77" t="inlineStr">
+        <is>
+          <t>SQL ready (ARWB_usp_SnapshotQueues); no nightly job scheduled yet.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="68" t="n">
@@ -7425,6 +7843,16 @@
           <t>Moved before the first grid (was after the Work Queue and Claim Detail): Work Queue, My Work, Follow-Up, QA and Assignment all use it.</t>
         </is>
       </c>
+      <c r="O39" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P39" s="77" t="inlineStr">
+        <is>
+          <t>Shared DataTable: server-side sort / paging, CSV export, column visibility, row selection; shared Modal and Notice.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="68" t="n">
@@ -7484,6 +7912,16 @@
           <t>Moved with T041. Saved Views are per user, so they need the user / role model.</t>
         </is>
       </c>
+      <c r="O40" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P40" s="77" t="inlineStr">
+        <is>
+          <t>Saved Views built: GET/POST/PUT/DELETE /api/ar-workbench/saved-views over dbo.ARWB_SavedView (per user + screen, 50 max, one default). Save / apply / star default / delete control on Work Queue, My Work and Follow-Up Management; default view opens with the screen. Rules unit-tested.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="68" t="n">
@@ -7544,6 +7982,16 @@
           <t>Now after the data, rules and grid it is built on.</t>
         </is>
       </c>
+      <c r="O41" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P41" s="77" t="inlineStr">
+        <is>
+          <t>Denial &amp; AR Work Queue: claim listing with server paging.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="68" t="n">
@@ -7604,6 +8052,16 @@
           <t>Now after the queue engine, TFL and financial model that supply its columns.</t>
         </is>
       </c>
+      <c r="O42" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P42" s="77" t="inlineStr">
+        <is>
+          <t>Work Queue columns include Aging, Denial Category, TFL, Priority, AR Queue and Expected Payment (Revenue Expectation, sortable).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="68" t="n">
@@ -7664,6 +8122,16 @@
           <t>Moved from Claim Detail Workspace: filters cascade to the claim listing, so they belong to the Work Queue.</t>
         </is>
       </c>
+      <c r="O43" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P43" s="77" t="inlineStr">
+        <is>
+          <t>Work Queue multi-select filters (clinic, payer, panel, category, status, agent, priority, aging, queue), kept in the URL.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="68" t="n">
@@ -7723,6 +8191,16 @@
           <t>Moved from Claim Detail Workspace with T026.</t>
         </is>
       </c>
+      <c r="O44" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P44" s="77" t="inlineStr">
+        <is>
+          <t>Listing re-queries on every filter change; filter chips.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="68" t="n">
@@ -7782,6 +8260,16 @@
           <t>Moved from Log Follow-Up Note: assigning claims (checkbox, multiselect, agent picker) is a Work Queue action.</t>
         </is>
       </c>
+      <c r="O45" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P45" s="77" t="inlineStr">
+        <is>
+          <t>Work Queue checkbox selection + Assign Selected (agent picker, note, due date).</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="68" t="n">
@@ -7841,6 +8329,16 @@
           <t>Moved from Log Follow-Up Note: export of the (scoped) claim listing.</t>
         </is>
       </c>
+      <c r="O46" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P46" s="77" t="inlineStr">
+        <is>
+          <t>Work Queue: Export Filtered / Export All to Excel - every matching claim in the caller's scope (up to 100,000 rows), not just the page.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="68" t="n">
@@ -7900,6 +8398,16 @@
           <t>Moved after the Work Queue: the drill-through lands on it.</t>
         </is>
       </c>
+      <c r="O47" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P47" s="77" t="inlineStr">
+        <is>
+          <t>Data Processing screen: Denial Analysis Report for the current and previous sync week (open claims / balance, top payer, impact, observation, action) with Route to Work Queue.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="68" t="n">
@@ -7959,6 +8467,16 @@
           <t>Moved after the Work Queue: the redirect lands on it.</t>
         </is>
       </c>
+      <c r="O48" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P48" s="77" t="inlineStr">
+        <is>
+          <t>Dashboard insights route to the Work Queue filtered to the denial code.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="68" t="n">
@@ -8019,6 +8537,16 @@
           <t>Now after the Work Queue it opens from and the activity tables its timeline reads.</t>
         </is>
       </c>
+      <c r="O49" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P49" s="77" t="inlineStr">
+        <is>
+          <t>Claim workspace (/claims/:claimKey) with Overview, CPT, Denial, Follow-Ups, Activity Timeline.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="68" t="n">
@@ -8078,6 +8606,16 @@
           <t>Now after the masters, status rules and Claim Detail it lives in. Note: it auto-submits to QA; the QA queue is P2 (T059 / T060).</t>
         </is>
       </c>
+      <c r="O50" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P50" s="77" t="inlineStr">
+        <is>
+          <t>Log Follow-Up Note on the claim workspace: Comments Framework fields, root cause when Denied, fix options by claim status, CIP block; saving sends the claim to QA (POST claims/{key}/follow-ups).</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="64" t="n">
@@ -8133,6 +8671,16 @@
         </is>
       </c>
       <c r="N51" s="65" t="inlineStr"/>
+      <c r="O51" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P51" s="77" t="inlineStr">
+        <is>
+          <t>No bulk follow-up upload.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="68" t="n">
@@ -8192,6 +8740,16 @@
           <t>Now after assignment (T031) and the agent role (T049) it depends on.</t>
         </is>
       </c>
+      <c r="O52" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P52" s="77" t="inlineStr">
+        <is>
+          <t>My Work page built (/my-work): 9 quick-filter tiles from GET work-summary, search + payer/panel/category/priority/status/TFL + more filters, AR Queue, Fix/Resolution, Next Follow-Up columns, Log Follow-Up action. Agent sees own caseload (SQL scope).</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="64" t="n">
@@ -8247,6 +8805,16 @@
         </is>
       </c>
       <c r="N53" s="65" t="inlineStr"/>
+      <c r="O53" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P53" s="77" t="inlineStr">
+        <is>
+          <t>Follow-Up Management page built (/follow-up): IsFollowUpActionable queue, overdue/today styling on Next Follow-Up, Agent + Last Follow-Up columns, Log Follow-Up drops the claim off the list.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="64" t="n">
@@ -8302,6 +8870,16 @@
         </is>
       </c>
       <c r="N54" s="65" t="inlineStr"/>
+      <c r="O54" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P54" s="77" t="inlineStr">
+        <is>
+          <t>Tiles All Active / Overdue / Due Today / Upcoming / No Follow-Up Scheduled with live counts; click filters the list.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="64" t="n">
@@ -8357,6 +8935,16 @@
         </is>
       </c>
       <c r="N55" s="65" t="inlineStr"/>
+      <c r="O55" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P55" s="77" t="inlineStr">
+        <is>
+          <t>Search, all filters, TFL and Save View (T042) in place on Follow-Up Management.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="64" t="n">
@@ -8412,6 +9000,16 @@
         </is>
       </c>
       <c r="N56" s="65" t="inlineStr"/>
+      <c r="O56" s="76" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P56" s="77" t="inlineStr">
+        <is>
+          <t>Tile + filter bar + more filters combine into the server-side claim query; option lists are lab-wide, not yet narrowed by the other selections.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="64" t="n">
@@ -8467,6 +9065,16 @@
         </is>
       </c>
       <c r="N57" s="65" t="inlineStr"/>
+      <c r="O57" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P57" s="77" t="inlineStr">
+        <is>
+          <t>Claim ID / row opens claim detail (back returns to the page); Log Follow-Up opens the same follow-up modal as the Work Queue.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="68" t="n">
@@ -8526,6 +9134,16 @@
           <t>Moved ahead of Assignment Management: the agent picker lists users with an agent role and lab access.</t>
         </is>
       </c>
+      <c r="O58" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P58" s="77" t="inlineStr">
+        <is>
+          <t>AR Workbench User Management page (/users) + GET/POST/PUT /api/ar-workbench/users: create with username, password, email, one AR Workbench role, multi-select labs; edit email/role/labs/active/password reset. Super Admin = all labs; AR Workbench System Administrator / Lab Admin = own dbo.UserLabs. Writes LRNMaster LabUsers/UserRoles/UserLabs in one transaction, LRN Metrics-compatible PBKDF2 hash. Own account, site admins and users with labs/roles outside the caller's reach are read-only. Clinic/Provider Viewer not offered (needs scope). Rules unit-tested.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="64" t="n">
@@ -8581,6 +9199,12 @@
         </is>
       </c>
       <c r="N59" s="65" t="inlineStr"/>
+      <c r="O59" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P59" s="77" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="64" t="n">
@@ -8636,6 +9260,16 @@
         </is>
       </c>
       <c r="N60" s="65" t="inlineStr"/>
+      <c r="O60" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P60" s="77" t="inlineStr">
+        <is>
+          <t>Assignment Management: Unassigned Claims (open balance, untouched 45+ days, Days Untouched).</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="64" t="n">
@@ -8691,6 +9325,16 @@
         </is>
       </c>
       <c r="N61" s="65" t="inlineStr"/>
+      <c r="O61" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P61" s="77" t="inlineStr">
+        <is>
+          <t>Create Assignment Batch (criteria preview, agent, due date) + Assignment Batches with live completion and running log.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="64" t="n">
@@ -8746,6 +9390,16 @@
         </is>
       </c>
       <c r="N62" s="65" t="inlineStr"/>
+      <c r="O62" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P62" s="77" t="inlineStr">
+        <is>
+          <t>Assigned Claims – Bulk Reassign + Agent Workload chart; reassigning resolves pending reassignment requests.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="68" t="n">
@@ -8805,6 +9459,16 @@
           <t>CHECK: same text as T048 ('Directing the user to Denial &amp; AR Queue for Followup log') — likely a copy; confirm the intended task.</t>
         </is>
       </c>
+      <c r="O63" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P63" s="77" t="inlineStr">
+        <is>
+          <t>Claims open in the claim workspace, where Log Follow-Up Note is now available.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="64" t="n">
@@ -8864,6 +9528,16 @@
           <t>No change. Start P2 with QA straight after P1 testing: follow-up notes auto-submit to QA from T029, so claims pile up in Submitted for QA until this lands.</t>
         </is>
       </c>
+      <c r="O64" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P64" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_ClaimQaReview table only.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="64" t="n">
@@ -8919,6 +9593,16 @@
         </is>
       </c>
       <c r="N65" s="65" t="inlineStr"/>
+      <c r="O65" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P65" s="77" t="inlineStr">
+        <is>
+          <t>QA Verification Queue is a planned page.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="64" t="n">
@@ -8978,6 +9662,16 @@
           <t>No change. A CIP case reaches Pending Approval only after QA approves the note (T059).</t>
         </is>
       </c>
+      <c r="O66" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P66" s="77" t="inlineStr">
+        <is>
+          <t>dbo.ARWB_CipCase / CipCaseHistory tables only.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="64" t="n">
@@ -9033,6 +9727,12 @@
         </is>
       </c>
       <c r="N67" s="65" t="inlineStr"/>
+      <c r="O67" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P67" s="77" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="64" t="n">
@@ -9088,6 +9788,12 @@
         </is>
       </c>
       <c r="N68" s="65" t="inlineStr"/>
+      <c r="O68" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P68" s="77" t="n"/>
     </row>
     <row r="69">
       <c r="B69" s="64" t="n">
@@ -9147,6 +9853,12 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O69" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P69" s="77" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="64" t="n">
@@ -9202,6 +9914,12 @@
         </is>
       </c>
       <c r="N70" s="65" t="inlineStr"/>
+      <c r="O70" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P70" s="77" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="64" t="n">
@@ -9257,6 +9975,12 @@
         </is>
       </c>
       <c r="N71" s="65" t="inlineStr"/>
+      <c r="O71" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P71" s="77" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="64" t="n">
@@ -9316,6 +10040,16 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O72" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P72" s="77" t="inlineStr">
+        <is>
+          <t>Per-claim Activity Timeline exists; no cross-claim Audit Logs screen.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="64" t="n">
@@ -9375,6 +10109,12 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O73" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P73" s="77" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="64" t="n">
@@ -9434,6 +10174,16 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O74" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P74" s="77" t="inlineStr">
+        <is>
+          <t>GET /api/ar-workbench/dashboard: 10 KPI tiles (claims, outstanding AR, unassigned, in progress, QA, completed, recovered, potential recovery, overdue follow-ups).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="64" t="n">
@@ -9489,6 +10239,16 @@
         </is>
       </c>
       <c r="N75" s="65" t="inlineStr"/>
+      <c r="O75" s="76" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="P75" s="77" t="inlineStr">
+        <is>
+          <t>Dashboard widgets: insights, AR Collections Progress, Queue Volumes, Category &amp; Aging, Workflow Status, Recovery Performance, Agent Productivity.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="64" t="n">
@@ -9548,6 +10308,12 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O76" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P76" s="77" t="n"/>
     </row>
     <row r="77">
       <c r="B77" s="64" t="n">
@@ -9603,6 +10369,12 @@
         </is>
       </c>
       <c r="N77" s="65" t="inlineStr"/>
+      <c r="O77" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P77" s="77" t="n"/>
     </row>
     <row r="78">
       <c r="B78" s="64" t="n">
@@ -9662,6 +10434,12 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O78" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P78" s="77" t="n"/>
     </row>
     <row r="79">
       <c r="B79" s="64" t="n">
@@ -9717,6 +10495,12 @@
         </is>
       </c>
       <c r="N79" s="65" t="inlineStr"/>
+      <c r="O79" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P79" s="77" t="n"/>
     </row>
     <row r="80">
       <c r="B80" s="64" t="n">
@@ -9772,6 +10556,12 @@
         </is>
       </c>
       <c r="N80" s="65" t="inlineStr"/>
+      <c r="O80" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P80" s="77" t="n"/>
     </row>
     <row r="81">
       <c r="B81" s="64" t="n">
@@ -9831,6 +10621,12 @@
           <t>No change.</t>
         </is>
       </c>
+      <c r="O81" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P81" s="77" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="64" t="n">
@@ -9886,6 +10682,12 @@
         </is>
       </c>
       <c r="N82" s="65" t="inlineStr"/>
+      <c r="O82" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P82" s="77" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="64" t="n">
@@ -9941,6 +10743,12 @@
         </is>
       </c>
       <c r="N83" s="65" t="inlineStr"/>
+      <c r="O83" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P83" s="77" t="n"/>
     </row>
     <row r="84">
       <c r="B84" s="64" t="n">
@@ -9996,6 +10804,12 @@
         </is>
       </c>
       <c r="N84" s="65" t="inlineStr"/>
+      <c r="O84" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P84" s="77" t="n"/>
     </row>
     <row r="85">
       <c r="B85" s="64" t="n">
@@ -10051,6 +10865,12 @@
         </is>
       </c>
       <c r="N85" s="65" t="inlineStr"/>
+      <c r="O85" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P85" s="77" t="n"/>
     </row>
     <row r="86">
       <c r="B86" s="64" t="n">
@@ -10106,6 +10926,12 @@
         </is>
       </c>
       <c r="N86" s="65" t="inlineStr"/>
+      <c r="O86" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P86" s="77" t="n"/>
     </row>
     <row r="87">
       <c r="B87" s="68" t="n">
@@ -10165,7 +10991,14 @@
           <t>Module ID was M23 (shared with Testing); Go-Live is its own module.</t>
         </is>
       </c>
-    </row>
+      <c r="O87" s="76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="P87" s="77" t="n"/>
+    </row>
+    <row r="88"/>
     <row r="89">
       <c r="B89" s="75" t="inlineStr">
         <is>
@@ -10194,16 +11027,304 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="B94" s="78" t="inlineStr">
+        <is>
+          <t>AR Workbench build status — as of 10/06/2026 (updated after the P1 follow-up work)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="79" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C95" s="79" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D95" s="79" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E95" s="79" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F95" s="79" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G95" s="79" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H95" s="79" t="inlineStr">
+        <is>
+          <t>% Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="80" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C96" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P0",$O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D96" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P0",$O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E96" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P0",$O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F96" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P0",$O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G96" s="81">
+        <f>SUM(C96:F96)</f>
+        <v/>
+      </c>
+      <c r="H96" s="82">
+        <f>IF(G96=0,0,C96/G96)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="80" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C97" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P1",$O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D97" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P1",$O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E97" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P1",$O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F97" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P1",$O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G97" s="81">
+        <f>SUM(C97:F97)</f>
+        <v/>
+      </c>
+      <c r="H97" s="82">
+        <f>IF(G97=0,0,C97/G97)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="80" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C98" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P2",$O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D98" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P2",$O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E98" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P2",$O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F98" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P2",$O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G98" s="81">
+        <f>SUM(C98:F98)</f>
+        <v/>
+      </c>
+      <c r="H98" s="82">
+        <f>IF(G98=0,0,C98/G98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="80" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C99" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P3",$O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D99" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P3",$O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E99" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P3",$O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F99" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P3",$O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G99" s="81">
+        <f>SUM(C99:F99)</f>
+        <v/>
+      </c>
+      <c r="H99" s="82">
+        <f>IF(G99=0,0,C99/G99)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="80" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C100" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P4",$O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D100" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P4",$O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E100" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P4",$O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F100" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P4",$O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G100" s="81">
+        <f>SUM(C100:F100)</f>
+        <v/>
+      </c>
+      <c r="H100" s="82">
+        <f>IF(G100=0,0,C100/G100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="80" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C101" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P5",$O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D101" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P5",$O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E101" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P5",$O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F101" s="80">
+        <f>COUNTIFS($H$6:$H$87,"P5",$O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G101" s="81">
+        <f>SUM(C101:F101)</f>
+        <v/>
+      </c>
+      <c r="H101" s="82">
+        <f>IF(G101=0,0,C101/G101)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="81" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C102" s="80">
+        <f>COUNTIF($O$6:$O$87,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D102" s="80">
+        <f>COUNTIF($O$6:$O$87,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="E102" s="80">
+        <f>COUNTIF($O$6:$O$87,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="F102" s="80">
+        <f>COUNTIF($O$6:$O$87,"Pending")</f>
+        <v/>
+      </c>
+      <c r="G102" s="81">
+        <f>SUM(C102:F102)</f>
+        <v/>
+      </c>
+      <c r="H102" s="82">
+        <f>IF(G102=0,0,C102/G102)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104" ht="30" customHeight="1">
+      <c r="B104" s="83" t="inlineStr">
+        <is>
+          <t>Completed = built in the AR Workbench (SQL + API + screen) and buildable; it is not UAT sign-off. In Progress = partly built (e.g. SQL ready, no screen or job yet). Not Started = nothing built. Pending = waiting on a business decision. Status column is a dropdown; the summary above recounts from it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B5:N87"/>
-  <mergeCells count="6">
+  <autoFilter ref="B5:P87"/>
+  <mergeCells count="7">
     <mergeCell ref="B90:N90"/>
+    <mergeCell ref="B104:N104"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B92:N92"/>
     <mergeCell ref="B91:N91"/>
     <mergeCell ref="B89:N89"/>
   </mergeCells>
+  <conditionalFormatting sqref="O6:O87">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Completed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Not Started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Pending"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="O6:O87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Completed, In Progress, Not Started or Pending." type="list">
+      <formula1>"Completed,In Progress,Not Started,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>